<commit_message>
Trazabilidad Ticket de Salida: registra respuestas de Clase 24b (Funciones - Uso del Retorno)
22 respuestas nuevas del 20/08/2026, incluyendo correccion de 9 filas
con tema generico mal emparejadas por el matcher de similitud.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015EJCYXwYS8FCJDkqunAYZW
</commit_message>
<xml_diff>
--- a/clases/Controles - Trazabilidad.xlsx
+++ b/clases/Controles - Trazabilidad.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1099,6 +1099,38 @@
         <v>2</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>25</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Control de Funciones</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Felipe Aravena Cárdenas</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>93</v>
+      </c>
+      <c r="F21" t="n">
+        <v>100</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="H21" t="n">
+        <v>6.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1110,7 +1142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1159,14 +1191,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Benjamín Díaz Silva</t>
+          <t>Felipe Aravena Cárdenas</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>2</v>
+        <v>6.6</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>6.6</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -1175,14 +1207,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cristóbal Muñoz Cubillos</t>
+          <t>Benjamín Díaz Silva</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>6.4</v>
+        <v>2</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -1191,14 +1223,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Damián Flores Silva</t>
+          <t>Cristóbal Muñoz Cubillos</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>2.6</v>
+        <v>6.4</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>6.4</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
@@ -1207,14 +1239,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Diego Cifuentes Tessada</t>
+          <t>Damián Flores Silva</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>2.6</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>2</v>
+        <v>2.6</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
@@ -1223,14 +1255,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Diego Donoso Figueroa</t>
+          <t>Diego Cifuentes Tessada</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3.7</v>
+        <v>2</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>3.7</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -1239,14 +1271,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Diego Peña Bustamante</t>
+          <t>Diego Donoso Figueroa</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>6.5</v>
+        <v>3.7</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>3.7</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
@@ -1255,14 +1287,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Diego Vargas Jaqui</t>
+          <t>Diego Peña Bustamante</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>2</v>
+        <v>6.5</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>6.5</v>
       </c>
       <c r="D9" t="n">
         <v>1</v>
@@ -1271,14 +1303,14 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Eduardo Pacco Ríos</t>
+          <t>Diego Vargas Jaqui</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>6.8</v>
+        <v>2</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
@@ -1287,14 +1319,14 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Felipe Román Brito</t>
+          <t>Eduardo Pacco Ríos</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6.3</v>
+        <v>6.8</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>6.3</v>
+        <v>6.8</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -1303,14 +1335,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Francisca Parra Marínquez</t>
+          <t>Felipe Román Brito</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>2.2</v>
+        <v>6.3</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>6.3</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -1319,14 +1351,14 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Francisco Vega Sanhueza</t>
+          <t>Francisca Parra Marínquez</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>2.2</v>
       </c>
       <c r="D13" t="n">
         <v>1</v>
@@ -1335,14 +1367,14 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Julián Aravena Sagal</t>
+          <t>Francisco Vega Sanhueza</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>3</v>
+        <v>6.8</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>6.8</v>
       </c>
       <c r="D14" t="n">
         <v>1</v>
@@ -1351,14 +1383,14 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Lucas Valenzuela Donoso</t>
+          <t>Julián Aravena Sagal</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3.9</v>
+        <v>3</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>3.9</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -1367,14 +1399,14 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Martín Sánchez Orellana</t>
+          <t>Lucas Valenzuela Donoso</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2.2</v>
+        <v>3.9</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>2.2</v>
+        <v>3.9</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
@@ -1383,14 +1415,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Maura Muñoz Gutiérrez</t>
+          <t>Martín Sánchez Orellana</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>6</v>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>6</v>
+        <v>2.2</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>2.2</v>
       </c>
       <c r="D17" t="n">
         <v>1</v>
@@ -1399,14 +1431,14 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Santino García Colombati</t>
+          <t>Maura Muñoz Gutiérrez</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D18" t="n">
         <v>1</v>
@@ -1415,14 +1447,14 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sebastián Ulloa Cuevas</t>
+          <t>Santino García Colombati</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4.3</v>
+        <v>7</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>4.3</v>
+        <v>7</v>
       </c>
       <c r="D19" t="n">
         <v>1</v>
@@ -1431,16 +1463,32 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>Sebastián Ulloa Cuevas</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Vicente Narváez Fernández</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B21" t="n">
         <v>2.8</v>
       </c>
-      <c r="C20" s="3" t="n">
+      <c r="C21" s="3" t="n">
         <v>2.8</v>
       </c>
-      <c r="D20" t="n">
+      <c r="D21" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1519,16 +1567,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E2" t="n">
-        <v>49.1</v>
+        <v>51.2</v>
       </c>
       <c r="F2" t="n">
-        <v>4.3</v>
+        <v>4.42</v>
       </c>
       <c r="G2" t="n">
-        <v>47.4</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert Controles - Trazabilidad.xlsx colado por accidente en el commit anterior
git add de las rutas de Tickets de Salida arrastro este archivo (ajeno a
esa tarea) por un lock de git concurrente en el momento del commit. Lo
devuelvo a su estado sin commitear para no mezclar el trabajo pendiente
de Controles con este cierre.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015EJCYXwYS8FCJDkqunAYZW
</commit_message>
<xml_diff>
--- a/clases/Controles - Trazabilidad.xlsx
+++ b/clases/Controles - Trazabilidad.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1099,38 +1099,6 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>25</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Control de Funciones</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Felipe Aravena Cárdenas</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>93</v>
-      </c>
-      <c r="F21" t="n">
-        <v>100</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="H21" t="n">
-        <v>6.6</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1142,7 +1110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1191,14 +1159,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Felipe Aravena Cárdenas</t>
+          <t>Benjamín Díaz Silva</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>6.6</v>
+        <v>2</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -1207,14 +1175,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Benjamín Díaz Silva</t>
+          <t>Cristóbal Muñoz Cubillos</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>2</v>
+        <v>6.4</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>6.4</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -1223,14 +1191,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cristóbal Muñoz Cubillos</t>
+          <t>Damián Flores Silva</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>6.4</v>
+        <v>2.6</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>2.6</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
@@ -1239,14 +1207,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Damián Flores Silva</t>
+          <t>Diego Cifuentes Tessada</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2.6</v>
+        <v>2</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>2.6</v>
+        <v>2</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
@@ -1255,14 +1223,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Diego Cifuentes Tessada</t>
+          <t>Diego Donoso Figueroa</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>3.7</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>2</v>
+        <v>3.7</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -1271,14 +1239,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Diego Donoso Figueroa</t>
+          <t>Diego Peña Bustamante</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>3.7</v>
+        <v>6.5</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>6.5</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
@@ -1287,14 +1255,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Diego Peña Bustamante</t>
+          <t>Diego Vargas Jaqui</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>6.5</v>
+        <v>2</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="D9" t="n">
         <v>1</v>
@@ -1303,14 +1271,14 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Diego Vargas Jaqui</t>
+          <t>Eduardo Pacco Ríos</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>2</v>
+        <v>6.8</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>6.8</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
@@ -1319,14 +1287,14 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Eduardo Pacco Ríos</t>
+          <t>Felipe Román Brito</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6.8</v>
+        <v>6.3</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>6.8</v>
+        <v>6.3</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -1335,14 +1303,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Felipe Román Brito</t>
+          <t>Francisca Parra Marínquez</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>6.3</v>
+        <v>2.2</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>2.2</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -1351,14 +1319,14 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Francisca Parra Marínquez</t>
+          <t>Francisco Vega Sanhueza</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>2.2</v>
+        <v>6.8</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>6.8</v>
       </c>
       <c r="D13" t="n">
         <v>1</v>
@@ -1367,14 +1335,14 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Francisco Vega Sanhueza</t>
+          <t>Julián Aravena Sagal</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>6.8</v>
+        <v>3</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="D14" t="n">
         <v>1</v>
@@ -1383,14 +1351,14 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Julián Aravena Sagal</t>
+          <t>Lucas Valenzuela Donoso</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>3.9</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>3</v>
+        <v>3.9</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -1399,14 +1367,14 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Lucas Valenzuela Donoso</t>
+          <t>Martín Sánchez Orellana</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3.9</v>
+        <v>2.2</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>3.9</v>
+        <v>2.2</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
@@ -1415,14 +1383,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Martín Sánchez Orellana</t>
+          <t>Maura Muñoz Gutiérrez</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="C17" s="3" t="n">
-        <v>2.2</v>
+        <v>6</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="D17" t="n">
         <v>1</v>
@@ -1431,14 +1399,14 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Maura Muñoz Gutiérrez</t>
+          <t>Santino García Colombati</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D18" t="n">
         <v>1</v>
@@ -1447,14 +1415,14 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Santino García Colombati</t>
+          <t>Sebastián Ulloa Cuevas</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>7</v>
+        <v>4.3</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>7</v>
+        <v>4.3</v>
       </c>
       <c r="D19" t="n">
         <v>1</v>
@@ -1463,32 +1431,16 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sebastián Ulloa Cuevas</t>
+          <t>Vicente Narváez Fernández</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="C20" s="2" t="n">
-        <v>4.3</v>
+        <v>2.8</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>2.8</v>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Vicente Narváez Fernández</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="C21" s="3" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="D21" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1567,16 +1519,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E2" t="n">
-        <v>51.2</v>
+        <v>49.1</v>
       </c>
       <c r="F2" t="n">
-        <v>4.42</v>
+        <v>4.3</v>
       </c>
       <c r="G2" t="n">
-        <v>50</v>
+        <v>47.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clase 28-32: split Strings en 3 clases + su lunes estándar, renumeración completa
Se separa el recorrido de cadenas con for en una clase nueva (N°29) para no
diluir el foco de indexing/slicing en N°28, y se agrega su propio lunes
estándar de control (N°31) — corriendo +2 todo lo posterior (Listas,
integración, Evaluación F+S+L, proyectos OA4/OA5). Bloque de Strings
adelantado al 31-ago. Historial-Curricular.md y Plan Cierre actualizados;
Prompt.md de cada clase con el contenido/objetivo acordado en la sesión de
diseño.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clases/Controles - Trazabilidad.xlsx
+++ b/clases/Controles - Trazabilidad.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1099,6 +1099,38 @@
         <v>2</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>25</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Control de Funciones</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Felipe Aravena Cárdenas</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>93</v>
+      </c>
+      <c r="F21" t="n">
+        <v>100</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="H21" t="n">
+        <v>6.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1110,7 +1142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1159,14 +1191,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Benjamín Díaz Silva</t>
+          <t>Felipe Aravena Cárdenas</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>2</v>
+        <v>6.6</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>6.6</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -1175,14 +1207,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cristóbal Muñoz Cubillos</t>
+          <t>Benjamín Díaz Silva</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>6.4</v>
+        <v>2</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -1191,14 +1223,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Damián Flores Silva</t>
+          <t>Cristóbal Muñoz Cubillos</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>2.6</v>
+        <v>6.4</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>6.4</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
@@ -1207,14 +1239,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Diego Cifuentes Tessada</t>
+          <t>Damián Flores Silva</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>2.6</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>2</v>
+        <v>2.6</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
@@ -1223,14 +1255,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Diego Donoso Figueroa</t>
+          <t>Diego Cifuentes Tessada</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3.7</v>
+        <v>2</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>3.7</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -1239,14 +1271,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Diego Peña Bustamante</t>
+          <t>Diego Donoso Figueroa</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>6.5</v>
+        <v>3.7</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>3.7</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
@@ -1255,14 +1287,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Diego Vargas Jaqui</t>
+          <t>Diego Peña Bustamante</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>2</v>
+        <v>6.5</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>6.5</v>
       </c>
       <c r="D9" t="n">
         <v>1</v>
@@ -1271,14 +1303,14 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Eduardo Pacco Ríos</t>
+          <t>Diego Vargas Jaqui</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>6.8</v>
+        <v>2</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
@@ -1287,14 +1319,14 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Felipe Román Brito</t>
+          <t>Eduardo Pacco Ríos</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6.3</v>
+        <v>6.8</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>6.3</v>
+        <v>6.8</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -1303,14 +1335,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Francisca Parra Marínquez</t>
+          <t>Felipe Román Brito</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>2.2</v>
+        <v>6.3</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>6.3</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -1319,14 +1351,14 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Francisco Vega Sanhueza</t>
+          <t>Francisca Parra Marínquez</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>2.2</v>
       </c>
       <c r="D13" t="n">
         <v>1</v>
@@ -1335,14 +1367,14 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Julián Aravena Sagal</t>
+          <t>Francisco Vega Sanhueza</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>3</v>
+        <v>6.8</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>6.8</v>
       </c>
       <c r="D14" t="n">
         <v>1</v>
@@ -1351,14 +1383,14 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Lucas Valenzuela Donoso</t>
+          <t>Julián Aravena Sagal</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3.9</v>
+        <v>3</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>3.9</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -1367,14 +1399,14 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Martín Sánchez Orellana</t>
+          <t>Lucas Valenzuela Donoso</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2.2</v>
+        <v>3.9</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>2.2</v>
+        <v>3.9</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
@@ -1383,14 +1415,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Maura Muñoz Gutiérrez</t>
+          <t>Martín Sánchez Orellana</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>6</v>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>6</v>
+        <v>2.2</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>2.2</v>
       </c>
       <c r="D17" t="n">
         <v>1</v>
@@ -1399,14 +1431,14 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Santino García Colombati</t>
+          <t>Maura Muñoz Gutiérrez</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D18" t="n">
         <v>1</v>
@@ -1415,14 +1447,14 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sebastián Ulloa Cuevas</t>
+          <t>Santino García Colombati</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4.3</v>
+        <v>7</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>4.3</v>
+        <v>7</v>
       </c>
       <c r="D19" t="n">
         <v>1</v>
@@ -1431,16 +1463,32 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>Sebastián Ulloa Cuevas</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Vicente Narváez Fernández</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B21" t="n">
         <v>2.8</v>
       </c>
-      <c r="C20" s="3" t="n">
+      <c r="C21" s="3" t="n">
         <v>2.8</v>
       </c>
-      <c r="D20" t="n">
+      <c r="D21" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1519,16 +1567,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E2" t="n">
-        <v>49.1</v>
+        <v>51.2</v>
       </c>
       <c r="F2" t="n">
-        <v>4.3</v>
+        <v>4.42</v>
       </c>
       <c r="G2" t="n">
-        <v>47.4</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>